<commit_message>
feat: label the VAT number as Matricule fiscal in the default templates
</commit_message>
<xml_diff>
--- a/db/templates/inbound_delivery_default.xlsx
+++ b/db/templates/inbound_delivery_default.xlsx
@@ -29,7 +29,7 @@
     <t>{{vendor.postalCode}} {{vendor.city}}</t>
   </si>
   <si>
-    <t>VAT: {{vendor.vatin}}</t>
+    <t>Matricule fiscal: {{vendor.vatin}}</t>
   </si>
   <si>
     <t>{{vendor.email}} | {{vendor.phone}}</t>
@@ -65,7 +65,7 @@
     <t>{{organization.postalCode}} {{organization.city}}</t>
   </si>
   <si>
-    <t>VAT: {{organization.vatin}}</t>
+    <t>Matricule fiscal: {{organization.vatin}}</t>
   </si>
   <si>
     <t>Product</t>

</xml_diff>